<commit_message>
Fix Excel catalogue loading and cart controls
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R334fdeebbf554776"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Guide" sheetId="2" r:id="Rb48ac78c03bd458e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R8956a3fac4634036"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Guide" sheetId="2" r:id="R4a979004f7b74e7e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -187,7 +187,7 @@
         <x:color rgb="FF842029"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFF8D7DA"/>
         </x:patternFill>
       </x:fill>
@@ -197,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ProductsTable" displayName="ProductsTable" ref="A1:Q8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="17">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ProductsTable" displayName="ProductsTable" ref="A1:R8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="18">
     <x:tableColumn id="1" name="id"/>
     <x:tableColumn id="2" name="active"/>
     <x:tableColumn id="3" name="name_en"/>
@@ -212,10 +212,11 @@
     <x:tableColumn id="11" name="description_en"/>
     <x:tableColumn id="12" name="description_te"/>
     <x:tableColumn id="13" name="material"/>
-    <x:tableColumn id="14" name="weave"/>
-    <x:tableColumn id="15" name="colour"/>
-    <x:tableColumn id="16" name="availability"/>
-    <x:tableColumn id="17" name="product_note"/>
+    <x:tableColumn id="14" name="yarn_count"/>
+    <x:tableColumn id="15" name="weave"/>
+    <x:tableColumn id="16" name="colour"/>
+    <x:tableColumn id="17" name="availability"/>
+    <x:tableColumn id="18" name="product_note"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -433,6 +434,7 @@
     <x:col min="15" max="15" width="25" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="25" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="25" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -476,15 +478,18 @@
         <x:v>material</x:v>
       </x:c>
       <x:c r="N1" s="9" t="str">
+        <x:v>yarn_count</x:v>
+      </x:c>
+      <x:c r="O1" s="9" t="str">
         <x:v>weave</x:v>
       </x:c>
-      <x:c r="O1" s="9" t="str">
+      <x:c r="P1" s="9" t="str">
         <x:v>colour</x:v>
       </x:c>
-      <x:c r="P1" s="9" t="str">
+      <x:c r="Q1" s="9" t="str">
         <x:v>availability</x:v>
       </x:c>
-      <x:c r="Q1" s="10" t="str">
+      <x:c r="R1" s="10" t="str">
         <x:v>product_note</x:v>
       </x:c>
     </x:row>
@@ -529,15 +534,18 @@
         <x:v>Hand-spun cotton</x:v>
       </x:c>
       <x:c r="N2" s="5" t="str">
+        <x:v>100 count</x:v>
+      </x:c>
+      <x:c r="O2" s="5" t="str">
         <x:v>Plain</x:v>
       </x:c>
-      <x:c r="O2" s="5" t="str">
+      <x:c r="P2" s="5" t="str">
         <x:v>Natural ivory</x:v>
       </x:c>
-      <x:c r="P2" s="5" t="str">
+      <x:c r="Q2" s="5" t="str">
         <x:v>In stock</x:v>
       </x:c>
-      <x:c r="Q2" s="12" t="str">
+      <x:c r="R2" s="12" t="str">
         <x:v>Fine counts and custom weaving are subject to current production.</x:v>
       </x:c>
     </x:row>
@@ -582,15 +590,18 @@
         <x:v>Hand-spun cotton</x:v>
       </x:c>
       <x:c r="N3" s="5" t="str">
+        <x:v>90 count</x:v>
+      </x:c>
+      <x:c r="O3" s="5" t="str">
         <x:v>Plain or bordered</x:v>
       </x:c>
-      <x:c r="O3" s="5" t="str">
+      <x:c r="P3" s="5" t="str">
         <x:v>Natural and dyed options</x:v>
       </x:c>
-      <x:c r="P3" s="5" t="str">
+      <x:c r="Q3" s="5" t="str">
         <x:v>In stock</x:v>
       </x:c>
-      <x:c r="Q3" s="12" t="str">
+      <x:c r="R3" s="12" t="str">
         <x:v>Ask AFKKS about current borders, colours and fine counts.</x:v>
       </x:c>
     </x:row>
@@ -635,15 +646,18 @@
         <x:v>Hand-spun cotton</x:v>
       </x:c>
       <x:c r="N4" s="5" t="str">
+        <x:v>100 count</x:v>
+      </x:c>
+      <x:c r="O4" s="5" t="str">
         <x:v>Plain or temple border</x:v>
       </x:c>
-      <x:c r="O4" s="5" t="str">
+      <x:c r="P4" s="5" t="str">
         <x:v>Natural ivory</x:v>
       </x:c>
-      <x:c r="P4" s="5" t="str">
+      <x:c r="Q4" s="5" t="str">
         <x:v>In stock</x:v>
       </x:c>
-      <x:c r="Q4" s="12" t="str">
+      <x:c r="R4" s="12" t="str">
         <x:v>Current options depend on loom availability.</x:v>
       </x:c>
     </x:row>
@@ -688,15 +702,18 @@
         <x:v>Hand-spun cotton</x:v>
       </x:c>
       <x:c r="N5" s="5" t="str">
+        <x:v>90 count</x:v>
+      </x:c>
+      <x:c r="O5" s="5" t="str">
         <x:v>Plain</x:v>
       </x:c>
-      <x:c r="O5" s="5" t="str">
+      <x:c r="P5" s="5" t="str">
         <x:v>White, cream and natural</x:v>
       </x:c>
-      <x:c r="P5" s="5" t="str">
+      <x:c r="Q5" s="5" t="str">
         <x:v>In stock</x:v>
       </x:c>
-      <x:c r="Q5" s="12" t="str">
+      <x:c r="R5" s="12" t="str">
         <x:v>Ask about current colours and counts.</x:v>
       </x:c>
     </x:row>
@@ -741,15 +758,18 @@
         <x:v>Cotton</x:v>
       </x:c>
       <x:c r="N6" s="5" t="str">
+        <x:v>40 count</x:v>
+      </x:c>
+      <x:c r="O6" s="5" t="str">
         <x:v>Absorbent handwoven cloth</x:v>
       </x:c>
-      <x:c r="O6" s="5" t="str">
+      <x:c r="P6" s="5" t="str">
         <x:v>Natural and coloured</x:v>
       </x:c>
-      <x:c r="P6" s="5" t="str">
+      <x:c r="Q6" s="5" t="str">
         <x:v>In stock</x:v>
       </x:c>
-      <x:c r="Q6" s="12" t="str">
+      <x:c r="R6" s="12" t="str">
         <x:v>Ask about bath towels, face towels and traditional gamchas.</x:v>
       </x:c>
     </x:row>
@@ -794,15 +814,18 @@
         <x:v>Hand-spun cotton</x:v>
       </x:c>
       <x:c r="N7" s="5" t="str">
+        <x:v>80 count</x:v>
+      </x:c>
+      <x:c r="O7" s="5" t="str">
         <x:v>Plain or bordered</x:v>
       </x:c>
-      <x:c r="O7" s="5" t="str">
+      <x:c r="P7" s="5" t="str">
         <x:v>Natural ivory</x:v>
       </x:c>
-      <x:c r="P7" s="5" t="str">
+      <x:c r="Q7" s="5" t="str">
         <x:v>In stock</x:v>
       </x:c>
-      <x:c r="Q7" s="12" t="str">
+      <x:c r="R7" s="12" t="str">
         <x:v>Made-to-order options may be available.</x:v>
       </x:c>
     </x:row>
@@ -847,15 +870,18 @@
         <x:v>Cotton or khadi blend</x:v>
       </x:c>
       <x:c r="N8" s="14" t="str">
+        <x:v>20 count</x:v>
+      </x:c>
+      <x:c r="O8" s="14" t="str">
         <x:v>Handwoven</x:v>
       </x:c>
-      <x:c r="O8" s="14" t="str">
+      <x:c r="P8" s="14" t="str">
         <x:v>Seasonal range</x:v>
       </x:c>
-      <x:c r="P8" s="14" t="str">
+      <x:c r="Q8" s="14" t="str">
         <x:v>Out of stock</x:v>
       </x:c>
-      <x:c r="Q8" s="17" t="str">
+      <x:c r="R8" s="17" t="str">
         <x:v>Materials, sizes and production require confirmation with AFKKS.</x:v>
       </x:c>
     </x:row>
@@ -875,7 +901,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fe84771c3f94e48"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64c331530a484d75"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>